<commit_message>
Already Created the Database with 4 tables, and uploaded it to google drive
</commit_message>
<xml_diff>
--- a/MiniProject/docs/data_dictionary.xlsx
+++ b/MiniProject/docs/data_dictionary.xlsx
@@ -8,12 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DEPI\Projects\Project\DEPI-ITC-ONL5-DA-Team3-G3-Projects\MiniProject\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BBB295A-C17B-4BF7-9E04-1EF0C41B30FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88ECBCC5-538C-41DA-BB79-C3665877FA86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example" sheetId="1" r:id="rId1"/>
+    <sheet name="Customers" sheetId="2" r:id="rId2"/>
+    <sheet name="Orders" sheetId="3" r:id="rId3"/>
+    <sheet name="Order Items" sheetId="4" r:id="rId4"/>
+    <sheet name="Products" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="129">
   <si>
     <t>Table</t>
   </si>
@@ -103,13 +107,337 @@
   <si>
     <t>PK
 Str</t>
+  </si>
+  <si>
+    <t>source_table</t>
+  </si>
+  <si>
+    <t>column_name</t>
+  </si>
+  <si>
+    <t>olist_orders_dataset</t>
+  </si>
+  <si>
+    <t>e481f51cbdc54678b7cc49136f2d6af7</t>
+  </si>
+  <si>
+    <t>53cdb2fc8bc7dce0b6741e2150273451</t>
+  </si>
+  <si>
+    <t>47770eb9100c2d0c44946d9cf07ec65d</t>
+  </si>
+  <si>
+    <t>9ef432eb6251297304e76186b10a928d</t>
+  </si>
+  <si>
+    <t>b0830fb4747a6c6d20dea0b8c802d7ef</t>
+  </si>
+  <si>
+    <t>41ce2a54c0b03bf3443c3d931a367089</t>
+  </si>
+  <si>
+    <t>order_status</t>
+  </si>
+  <si>
+    <t>delivered</t>
+  </si>
+  <si>
+    <t>order_purchase_timestamp</t>
+  </si>
+  <si>
+    <t>order_approved_at</t>
+  </si>
+  <si>
+    <t>order_delivered_carrier_date</t>
+  </si>
+  <si>
+    <t>order_delivered_customer_date</t>
+  </si>
+  <si>
+    <t>order_estimated_delivery_date</t>
+  </si>
+  <si>
+    <t>olist_products_dataset</t>
+  </si>
+  <si>
+    <t>Sample_1</t>
+  </si>
+  <si>
+    <t>Sample_2</t>
+  </si>
+  <si>
+    <t>Sample_3</t>
+  </si>
+  <si>
+    <t>1e9e8ef04dbcff4541ed26657ea517e5</t>
+  </si>
+  <si>
+    <t>3aa071139cb16b67ca9e5dea641aaa2f</t>
+  </si>
+  <si>
+    <t>96bd76ec8810374ed1b65e291975717f</t>
+  </si>
+  <si>
+    <t>product_category_name</t>
+  </si>
+  <si>
+    <t>perfumaria</t>
+  </si>
+  <si>
+    <t>artes</t>
+  </si>
+  <si>
+    <t>esporte_lazer</t>
+  </si>
+  <si>
+    <t>product_name_lenght</t>
+  </si>
+  <si>
+    <t>product_description_lenght</t>
+  </si>
+  <si>
+    <t>product_photos_qty</t>
+  </si>
+  <si>
+    <t>product_weight_g</t>
+  </si>
+  <si>
+    <t>product_length_cm</t>
+  </si>
+  <si>
+    <t>product_height_cm</t>
+  </si>
+  <si>
+    <t>product_width_cm</t>
+  </si>
+  <si>
+    <t>payment_sequential</t>
+  </si>
+  <si>
+    <t>payment_type</t>
+  </si>
+  <si>
+    <t>payment_installments</t>
+  </si>
+  <si>
+    <t>payment_value</t>
+  </si>
+  <si>
+    <t>b81ef226f3fe1789b1e8b2acac839d17</t>
+  </si>
+  <si>
+    <t>credit_card</t>
+  </si>
+  <si>
+    <t>a9810da82917af2d9aefd1278f1dcfa0</t>
+  </si>
+  <si>
+    <t>25e8ea4e93396b6fa0d3dd708e76c1bd</t>
+  </si>
+  <si>
+    <t>olist_order_payments_dataset</t>
+  </si>
+  <si>
+    <t>product_category_name_translati</t>
+  </si>
+  <si>
+    <t>product_category_name_english</t>
+  </si>
+  <si>
+    <t>beleza_saude</t>
+  </si>
+  <si>
+    <t>health_beauty</t>
+  </si>
+  <si>
+    <t>informatica_acessorios</t>
+  </si>
+  <si>
+    <t>computers_accessories</t>
+  </si>
+  <si>
+    <t>automotivo</t>
+  </si>
+  <si>
+    <t>auto</t>
+  </si>
+  <si>
+    <t>olist_order_items_dataset</t>
+  </si>
+  <si>
+    <t>00010242fe8c5a6d1ba2dd792cb16214</t>
+  </si>
+  <si>
+    <t>00018f77f2f0320c557190d7a144bdd3</t>
+  </si>
+  <si>
+    <t>000229ec398224ef6ca0657da4fc703e</t>
+  </si>
+  <si>
+    <t>order_item_id</t>
+  </si>
+  <si>
+    <t>4244733e06e7ecb4970a6e2683c13e61</t>
+  </si>
+  <si>
+    <t>e5f2d52b802189ee658865ca93d83a8f</t>
+  </si>
+  <si>
+    <t>c777355d18b72b67abbeef9df44fd0fd</t>
+  </si>
+  <si>
+    <t>seller_id</t>
+  </si>
+  <si>
+    <t>48436dade18ac8b2bce089ec2a041202</t>
+  </si>
+  <si>
+    <t>dd7ddc04e1b6c2c614352b383efe2d36</t>
+  </si>
+  <si>
+    <t>5b51032eddd242adc84c38acab88f23d</t>
+  </si>
+  <si>
+    <t>shipping_limit_date</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>freight_value</t>
+  </si>
+  <si>
+    <t>review_id</t>
+  </si>
+  <si>
+    <t>7bc2406110b926393aa56f80a40eba40</t>
+  </si>
+  <si>
+    <t>80e641a11e56f04c1ad469d5645fdfde</t>
+  </si>
+  <si>
+    <t>228ce5500dc1d8e020d8d1322874b6f0</t>
+  </si>
+  <si>
+    <t>73fc7af87114b39712e6da79b0a377eb</t>
+  </si>
+  <si>
+    <t>a548910a1c6147796b98fdf73dbeba33</t>
+  </si>
+  <si>
+    <t>f9e4b658b201a9f2ecdecbb34bed034b</t>
+  </si>
+  <si>
+    <t>review_score</t>
+  </si>
+  <si>
+    <t>review_comment_title</t>
+  </si>
+  <si>
+    <t>review_comment_message</t>
+  </si>
+  <si>
+    <t>olist_order_reviews_dataset</t>
+  </si>
+  <si>
+    <t>olist_customers_dataset</t>
+  </si>
+  <si>
+    <t>06b8999e2fba1a1fbc88172c00ba8bc7</t>
+  </si>
+  <si>
+    <t>18955e83d337fd6b2def6b18a428ac77</t>
+  </si>
+  <si>
+    <t>4e7b3e00288586ebd08712fdd0374a03</t>
+  </si>
+  <si>
+    <t>customer_unique_id</t>
+  </si>
+  <si>
+    <t>861eff4711a542e4b93843c6dd7febb0</t>
+  </si>
+  <si>
+    <t>290c77bc529b7ac935b93aa66c333dc3</t>
+  </si>
+  <si>
+    <t>060e732b5b29e8181a18229c7b0b2b5e</t>
+  </si>
+  <si>
+    <t>customer_zip_code_prefix</t>
+  </si>
+  <si>
+    <t>franca</t>
+  </si>
+  <si>
+    <t>sao bernardo do campo</t>
+  </si>
+  <si>
+    <t>sao paulo</t>
+  </si>
+  <si>
+    <t>customer_state</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>olist_geolocation_dataset</t>
+  </si>
+  <si>
+    <t>geolocation_zip_code_prefix</t>
+  </si>
+  <si>
+    <t>geolocation_lat</t>
+  </si>
+  <si>
+    <t>geolocation_lng</t>
+  </si>
+  <si>
+    <t>geolocation_city</t>
+  </si>
+  <si>
+    <t>geolocation_state</t>
+  </si>
+  <si>
+    <t>constraints</t>
+  </si>
+  <si>
+    <t>VARCHAR</t>
+  </si>
+  <si>
+    <t>DATETIME</t>
+  </si>
+  <si>
+    <t>INT</t>
+  </si>
+  <si>
+    <t>DECIMAL</t>
+  </si>
+  <si>
+    <t>REMOVE</t>
+  </si>
+  <si>
+    <t>NORMALIZATION PK KEY, VARCHAR</t>
+  </si>
+  <si>
+    <t>PK, VARCHAR</t>
+  </si>
+  <si>
+    <t>NORMALIZATION FK KEY, VARCHAR</t>
+  </si>
+  <si>
+    <t>FK, VARCHAR</t>
+  </si>
+  <si>
+    <t>NORMALIZATION KEY, VARCHAR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -124,6 +452,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -146,13 +486,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -558,4 +904,1063 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{587D8C5D-6B7C-424D-803E-ECB12A39A5B6}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="34.21875" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4">
+        <v>14409</v>
+      </c>
+      <c r="E4">
+        <v>9790</v>
+      </c>
+      <c r="F4">
+        <v>1151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E5" t="s">
+        <v>108</v>
+      </c>
+      <c r="F5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D7">
+        <v>1037</v>
+      </c>
+      <c r="E7">
+        <v>1046</v>
+      </c>
+      <c r="F7">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>122</v>
+      </c>
+      <c r="B8" t="s">
+        <v>112</v>
+      </c>
+      <c r="C8" t="s">
+        <v>114</v>
+      </c>
+      <c r="D8">
+        <v>-23.545621281152599</v>
+      </c>
+      <c r="E8">
+        <v>-23.546081127035499</v>
+      </c>
+      <c r="F8">
+        <v>-23.546128966414599</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C9" t="s">
+        <v>115</v>
+      </c>
+      <c r="D9">
+        <v>-46.6392920480016</v>
+      </c>
+      <c r="E9">
+        <v>-46.644820298371499</v>
+      </c>
+      <c r="F9">
+        <v>-46.642951483611299</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D10" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" t="s">
+        <v>109</v>
+      </c>
+      <c r="F10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D11" t="s">
+        <v>111</v>
+      </c>
+      <c r="E11" t="s">
+        <v>111</v>
+      </c>
+      <c r="F11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{859C17F7-BA5D-4D76-A070-7A0FC7558375}">
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="3">
+        <v>43010.455937500003</v>
+      </c>
+      <c r="E5" s="3">
+        <v>43305.862233796295</v>
+      </c>
+      <c r="F5" s="3">
+        <v>43320.360289351855</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="3">
+        <v>43010.463368055556</v>
+      </c>
+      <c r="E6" s="3">
+        <v>43307.141979166663</v>
+      </c>
+      <c r="F6" s="3">
+        <v>43320.371793981481</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="3">
+        <v>43012.829861111109</v>
+      </c>
+      <c r="E7" s="3">
+        <v>43307.604861111111</v>
+      </c>
+      <c r="F7" s="3">
+        <v>43320.576388888891</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="3">
+        <v>43018.892511574071</v>
+      </c>
+      <c r="E8" s="3">
+        <v>43319.644270833334</v>
+      </c>
+      <c r="F8" s="3">
+        <v>43329.754502314812</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="3">
+        <v>43026</v>
+      </c>
+      <c r="E9" s="3">
+        <v>43325</v>
+      </c>
+      <c r="F9" s="3">
+        <v>43347</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="B10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" t="s">
+        <v>61</v>
+      </c>
+      <c r="F10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>121</v>
+      </c>
+      <c r="B13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13">
+        <v>8</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>122</v>
+      </c>
+      <c r="B14" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14">
+        <v>99.33</v>
+      </c>
+      <c r="E14">
+        <v>24.39</v>
+      </c>
+      <c r="F14">
+        <v>65.709999999999994</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>119</v>
+      </c>
+      <c r="B15" t="s">
+        <v>97</v>
+      </c>
+      <c r="C15" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" t="s">
+        <v>88</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="F15" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="B16" t="s">
+        <v>97</v>
+      </c>
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" t="s">
+        <v>91</v>
+      </c>
+      <c r="E16" t="s">
+        <v>92</v>
+      </c>
+      <c r="F16" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" t="s">
+        <v>97</v>
+      </c>
+      <c r="C17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17">
+        <v>4</v>
+      </c>
+      <c r="E17">
+        <v>5</v>
+      </c>
+      <c r="F17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>119</v>
+      </c>
+      <c r="B18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C18" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>119</v>
+      </c>
+      <c r="B19" t="s">
+        <v>97</v>
+      </c>
+      <c r="C19" t="s">
+        <v>96</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61AFDB72-BE4D-4728-B556-A9449C5BF07B}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="32.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="3">
+        <v>42997.406655092593</v>
+      </c>
+      <c r="E6" s="3">
+        <v>42858.461956018517</v>
+      </c>
+      <c r="F6" s="3">
+        <v>43118.617013888892</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7">
+        <v>58.9</v>
+      </c>
+      <c r="E7">
+        <v>239.9</v>
+      </c>
+      <c r="F7">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>122</v>
+      </c>
+      <c r="B8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8">
+        <v>13.29</v>
+      </c>
+      <c r="E8">
+        <v>19.93</v>
+      </c>
+      <c r="F8">
+        <v>17.87</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AC822C8-8C2E-4DED-9048-3425C6D6DA85}">
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="39.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>122</v>
+      </c>
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4">
+        <v>40</v>
+      </c>
+      <c r="E4">
+        <v>44</v>
+      </c>
+      <c r="F4">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>287</v>
+      </c>
+      <c r="E5">
+        <v>276</v>
+      </c>
+      <c r="F5">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7">
+        <v>225</v>
+      </c>
+      <c r="E7">
+        <v>1000</v>
+      </c>
+      <c r="F7">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>122</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8">
+        <v>16</v>
+      </c>
+      <c r="E8">
+        <v>30</v>
+      </c>
+      <c r="F8">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
+      <c r="E9">
+        <v>18</v>
+      </c>
+      <c r="F9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>122</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10">
+        <v>14</v>
+      </c>
+      <c r="E10">
+        <v>20</v>
+      </c>
+      <c r="F10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>